<commit_message>
update excel dashboard and data analysis
</commit_message>
<xml_diff>
--- a/arkham-games-dataset.xlsx
+++ b/arkham-games-dataset.xlsx
@@ -2,25 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a35c853927159e38/Desktop/Projetos de Análise de Dados/Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{213CE9CF-7CEC-4187-B12A-586AD60CA2C4}"/>
-  <workbookProtection lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="450" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A675095C-2E64-4EFF-843A-09CAB47D6FA5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{D6B36053-BC7E-4879-83CB-ED370B1714CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D6B36053-BC7E-4879-83CB-ED370B1714CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados" sheetId="9" r:id="rId1"/>
-    <sheet name="TD" sheetId="18" r:id="rId2"/>
+    <sheet name="Tabela Dinâmica" sheetId="18" r:id="rId2"/>
     <sheet name="Dashboard" sheetId="11" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <pivotCaches>
-    <pivotCache cacheId="15" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -105,11 +104,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,24 +119,43 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -149,59 +168,313 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFC4C7C5"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </left>
       <right style="medium">
-        <color rgb="FFC4C7C5"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </right>
       <top style="medium">
-        <color rgb="FFC4C7C5"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </top>
       <bottom style="medium">
-        <color rgb="FFC4C7C5"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="32">
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </left>
+        <right style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </right>
+        <top style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="medium">
+          <color theme="0" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3" tint="9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3" tint="9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3" tint="9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3" tint="9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="0.0"/>
@@ -479,7 +752,7 @@
                 <c:pt idx="1">
                   <c:v>93.6</c:v>
                 </c:pt>
-                <c:pt idx="2" formatCode="0">
+                <c:pt idx="2">
                   <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="3">
@@ -812,13 +1085,13 @@
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="4"/>
-                <c:pt idx="0" formatCode="0">
+                <c:pt idx="0">
                   <c:v>86</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>87.6</c:v>
                 </c:pt>
-                <c:pt idx="2" formatCode="0">
+                <c:pt idx="2">
                   <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="3">
@@ -1214,7 +1487,7 @@
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="4"/>
-                <c:pt idx="0" formatCode="0">
+                <c:pt idx="0">
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="1">
@@ -1223,7 +1496,7 @@
                 <c:pt idx="2">
                   <c:v>12.5</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0">
+                <c:pt idx="3">
                   <c:v>17</c:v>
                 </c:pt>
               </c:numCache>
@@ -1439,7 +1712,7 @@
             <c:numRef>
               <c:f>Dados!$H$2:$H$5</c:f>
               <c:numCache>
-                <c:formatCode>0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>25</c:v>
@@ -1447,10 +1720,10 @@
                 <c:pt idx="1">
                   <c:v>45</c:v>
                 </c:pt>
-                <c:pt idx="2" formatCode="0.0">
+                <c:pt idx="2">
                   <c:v>41.5</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0.0">
+                <c:pt idx="3">
                   <c:v>51.5</c:v>
                 </c:pt>
               </c:numCache>
@@ -1542,7 +1815,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1692,48 +1965,6 @@
             </c:extLst>
           </c:dPt>
           <c:dLbls>
-            <c:dLbl>
-              <c:idx val="1"/>
-              <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                  <a:spAutoFit/>
-                </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="bg1"/>
-                      </a:solidFill>
-                      <a:latin typeface="Montserrat" panose="00000500000000000000" pitchFamily="2" charset="0"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="pt-BR"/>
-                </a:p>
-              </c:txPr>
-              <c:dLblPos val="ctr"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000007-34B2-4A4A-83A9-4F602FEEF50A}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
@@ -1789,7 +2020,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>TD!$A$2:$A$3</c:f>
+              <c:f>'Tabela Dinâmica'!$A$2:$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -1803,11 +2034,11 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>TD!$B$2:$B$3</c:f>
+              <c:f>'Tabela Dinâmica'!$B$2:$B$3</c:f>
               <c:numCache>
-                <c:formatCode>0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0" formatCode="0.0">
+                <c:pt idx="0">
                   <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
@@ -2107,19 +2338,19 @@
             <c:numRef>
               <c:f>Dados!$I$2:$I$5</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>6.7389999999999999</c:v>
+                  <c:v>6739</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.8710000000000004</c:v>
+                  <c:v>6871</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>25.016999999999999</c:v>
+                  <c:v>25017</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27.405999999999999</c:v>
+                  <c:v>27406</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2132,7 +2363,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -2213,7 +2443,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4555,7 +4785,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18067211" cy="8639342"/>
+          <a:ext cx="18130758" cy="8827394"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5092,10 +5322,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Giancarlo Lencioni de Castro" refreshedDate="46298.768877083334" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="4" xr:uid="{E5C783D3-0E5E-4336-83FE-FB6E1E4FDD59}">
   <cacheSource type="worksheet">
@@ -5142,7 +5368,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{03E154D3-6874-4D3F-AB50-BBF764B6DE64}" name="Tabela dinâmica5" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Desenvolvedora">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{03E154D3-6874-4D3F-AB50-BBF764B6DE64}" name="Tabela dinâmica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Desenvolvedora">
   <location ref="A1:B4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
@@ -5174,11 +5400,110 @@
   <dataFields count="1">
     <dataField name="Soma de Vendas (milhões)" fld="1" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="2">
-    <format dxfId="1">
+  <formats count="32">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="30">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="28">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="26">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="24">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="22">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="20">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="18">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="1">
@@ -5186,6 +5511,9 @@
           </reference>
         </references>
       </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -5517,165 +5845,168 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011BD3C3-1F40-4AD0-8E16-619C35E673D0}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="9" width="29.140625" style="2" customWidth="1"/>
+    <col min="1" max="9" width="29.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="9">
         <v>2009</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="10">
         <v>9.5</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="10">
         <v>91.3</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="10">
         <v>86</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="10">
         <v>12</v>
       </c>
-      <c r="H2" s="8">
+      <c r="H2" s="10">
         <v>25</v>
       </c>
-      <c r="I2" s="6">
-        <v>6.7389999999999999</v>
+      <c r="I2" s="11">
+        <v>6739</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2011</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>12.5</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="10">
         <v>93.6</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="10">
         <v>87.6</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="10">
         <v>12.5</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="10">
         <v>45</v>
       </c>
-      <c r="I3" s="6">
-        <v>6.8710000000000004</v>
+      <c r="I3" s="11">
+        <v>6871</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>2013</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>7</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="10">
         <v>73</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="10">
         <v>77</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="10">
         <v>12.5</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="10">
         <v>41.5</v>
       </c>
-      <c r="I4" s="6">
-        <v>25.016999999999999</v>
+      <c r="I4" s="11">
+        <v>25017</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>2015</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="10">
         <v>7.5</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="10">
         <v>80.599999999999994</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="10">
         <v>66.3</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>17</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="10">
         <v>51.5</v>
       </c>
-      <c r="I5" s="6">
-        <v>27.405999999999999</v>
+      <c r="I5" s="11">
+        <v>27406</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
 
@@ -5684,44 +6015,42 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="5">
         <v>29.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="5">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="6">
         <v>36.5</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -5731,7 +6060,6 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Apply final refinements to Excel workbook
Applied final polish and formatting adjustments to the Excel dataset and dashboard layout.
</commit_message>
<xml_diff>
--- a/arkham-games-dataset.xlsx
+++ b/arkham-games-dataset.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a35c853927159e38/Desktop/Projetos de Análise de Dados/Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="450" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A675095C-2E64-4EFF-843A-09CAB47D6FA5}"/>
+  <xr:revisionPtr revIDLastSave="580" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CCC6037-F89E-4F31-8AB6-20E34591E013}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D6B36053-BC7E-4879-83CB-ED370B1714CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{D6B36053-BC7E-4879-83CB-ED370B1714CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados" sheetId="9" r:id="rId1"/>
-    <sheet name="Tabela Dinâmica" sheetId="18" r:id="rId2"/>
+    <sheet name="Tabela_Dinâmica" sheetId="18" r:id="rId2"/>
     <sheet name="Dashboard" sheetId="11" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>Jogo</t>
   </si>
@@ -96,9 +96,6 @@
   <si>
     <t>Soma de Vendas (milhões)</t>
   </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
 </sst>
 </file>
 
@@ -106,8 +103,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -197,21 +194,21 @@
     <xf numFmtId="9" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -225,7 +222,7 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0"/>
+      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <font>
@@ -477,17 +474,17 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0"/>
+      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF8B1E2D"/>
+      <color rgb="FF26382F"/>
       <color rgb="FF1E3F5A"/>
-      <color rgb="FF8B1E2D"/>
       <color rgb="FF090A0C"/>
       <color rgb="FFD94A11"/>
-      <color rgb="FF26382F"/>
       <color rgb="FFE65100"/>
       <color rgb="FFE6E6E6"/>
       <color rgb="FF263A4A"/>
@@ -531,10 +528,10 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>NotaCríticos</c:v>
+            <c:v>Nota dos Críticos</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill flip="none" rotWithShape="1">
+            <a:gradFill>
               <a:gsLst>
                 <a:gs pos="100000">
                   <a:schemeClr val="bg1">
@@ -542,11 +539,10 @@
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="50000">
-                  <a:srgbClr val="1E3F5A"/>
+                  <a:srgbClr val="8B1E2D"/>
                 </a:gs>
               </a:gsLst>
               <a:lin ang="5400000" scaled="1"/>
-              <a:tileRect/>
             </a:gradFill>
             <a:ln>
               <a:solidFill>
@@ -573,7 +569,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -585,7 +581,6 @@
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -771,7 +766,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>NotaUsuários</c:v>
+            <c:v>Nota dos Usuários</c:v>
           </c:tx>
           <c:spPr>
             <a:gradFill>
@@ -839,7 +834,7 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="8B1E2D"/>
+                    <a:srgbClr val="1E3F5A"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
@@ -1223,6 +1218,34 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="Montserrat" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1288,7 +1311,7 @@
             <c:v>História</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill flip="none" rotWithShape="1">
+            <a:gradFill>
               <a:gsLst>
                 <a:gs pos="100000">
                   <a:schemeClr val="bg1">
@@ -1300,7 +1323,6 @@
                 </a:gs>
               </a:gsLst>
               <a:lin ang="10800000" scaled="1"/>
-              <a:tileRect/>
             </a:gradFill>
             <a:ln>
               <a:solidFill>
@@ -1315,7 +1337,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1327,7 +1349,6 @@
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1347,7 +1368,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1359,7 +1380,6 @@
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1379,7 +1399,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1387,11 +1407,10 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="8B1E2D"/>
+                    <a:srgbClr val="1E3F5A"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1515,7 +1534,7 @@
             <c:v>100%</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill flip="none" rotWithShape="1">
+            <a:gradFill>
               <a:gsLst>
                 <a:gs pos="100000">
                   <a:schemeClr val="bg1">
@@ -1523,11 +1542,10 @@
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="50000">
-                  <a:srgbClr val="1E3F5A"/>
+                  <a:srgbClr val="8B1E2D"/>
                 </a:gs>
               </a:gsLst>
               <a:lin ang="10800000" scaled="1"/>
-              <a:tileRect/>
             </a:gradFill>
             <a:ln>
               <a:solidFill>
@@ -1542,7 +1560,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1550,11 +1568,10 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1574,7 +1591,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1582,11 +1599,10 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1606,7 +1622,7 @@
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:gradFill flip="none" rotWithShape="1">
+              <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
                     <a:schemeClr val="bg1">
@@ -1618,7 +1634,6 @@
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="10800000" scaled="1"/>
-                <a:tileRect/>
               </a:gradFill>
               <a:ln>
                 <a:solidFill>
@@ -1855,6 +1870,34 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="Montserrat" panose="00000500000000000000" pitchFamily="2" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -2020,7 +2063,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Tabela Dinâmica'!$A$2:$A$3</c:f>
+              <c:f>Tabela_Dinâmica!$A$2:$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -2034,7 +2077,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Tabela Dinâmica'!$B$2:$B$3</c:f>
+              <c:f>Tabela_Dinâmica!$B$2:$B$3</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -2355,7 +2398,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-7FAB-45B6-B80C-90B75B930EBD}"/>
@@ -2434,8 +2477,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="bg1">
-                  <a:lumMod val="50000"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -4766,10 +4810,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>19843</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>153971</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>35294</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4785,7 +4829,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18130758" cy="8827394"/>
+          <a:ext cx="19260000" cy="9000000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4855,15 +4899,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>490942</xdr:colOff>
+      <xdr:colOff>490941</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>64461</xdr:rowOff>
+      <xdr:rowOff>90438</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>435773</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>311728</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>38529</xdr:rowOff>
+      <xdr:rowOff>64506</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4893,13 +4937,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>206572</xdr:colOff>
+      <xdr:colOff>491553</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>17900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>304062</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>311117</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>71031</xdr:rowOff>
     </xdr:to>
@@ -4916,8 +4960,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2612888" y="201716"/>
-          <a:ext cx="3706963" cy="420762"/>
+          <a:off x="2956847" y="204665"/>
+          <a:ext cx="4133829" cy="426660"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4952,7 +4996,7 @@
               </a:solidFill>
               <a:latin typeface="Montserrat" panose="00000500000000000000" pitchFamily="2" charset="0"/>
             </a:rPr>
-            <a:t>Notas Médias: Críticos e Usuários</a:t>
+            <a:t>Médias de Notas: Críticos e Usuários</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -4964,16 +5008,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>53476</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>267715</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>64461</xdr:rowOff>
+      <xdr:rowOff>90438</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>10203</xdr:colOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>224442</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>38529</xdr:rowOff>
+      <xdr:rowOff>64506</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5002,14 +5046,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>373568</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>449434</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>27457</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>577895</xdr:colOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>42722</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>61474</xdr:rowOff>
     </xdr:to>
@@ -5026,8 +5070,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11201989" y="211273"/>
-          <a:ext cx="5016959" cy="401648"/>
+          <a:off x="12159581" y="214222"/>
+          <a:ext cx="5140200" cy="407546"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5077,14 +5121,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>490942</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>428919</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>143162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>435773</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>373751</xdr:colOff>
       <xdr:row>45</xdr:row>
       <xdr:rowOff>117229</xdr:rowOff>
     </xdr:to>
@@ -5115,14 +5159,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>525206</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>370435</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>155496</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>587006</xdr:colOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>432235</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>76080</xdr:rowOff>
     </xdr:to>
@@ -5139,8 +5183,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1728364" y="4934707"/>
-          <a:ext cx="5476010" cy="472031"/>
+          <a:off x="2219406" y="5011378"/>
+          <a:ext cx="5608711" cy="480878"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5199,14 +5243,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>53476</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>267715</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>143162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>10203</xdr:colOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>224442</xdr:colOff>
       <xdr:row>45</xdr:row>
       <xdr:rowOff>117229</xdr:rowOff>
     </xdr:to>
@@ -5237,16 +5281,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>577359</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>42187</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>175415</xdr:rowOff>
+      <xdr:rowOff>175416</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>374104</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>449970</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>56160</xdr:rowOff>
+      <xdr:rowOff>56161</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5261,8 +5305,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11405780" y="4954626"/>
-          <a:ext cx="4609377" cy="432192"/>
+          <a:off x="12368658" y="5031298"/>
+          <a:ext cx="4722047" cy="441039"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5320,6 +5364,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5398,7 +5446,7 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Soma de Vendas (milhões)" fld="1" baseField="0" baseItem="0" numFmtId="165"/>
+    <dataField name="Soma de Vendas (milhões)" fld="1" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="32">
     <format dxfId="31">
@@ -5843,12 +5891,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{BE017181-E9CE-42C7-94B1-882A3C63FC95}">
+  <we:reference id="wa200010215" version="2.0.0.1" store="pt-BR" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200010215" version="2.0.0.1" store="wa200010215" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011BD3C3-1F40-4AD0-8E16-619C35E673D0}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="9" width="29.140625" style="1" customWidth="1"/>
@@ -5887,28 +5955,28 @@
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="9">
-        <v>2009</v>
+      <c r="B2" s="11">
+        <v>40050</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="9">
         <v>9.5</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="9">
         <v>91.3</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="9">
         <v>86</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="9">
         <v>12</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="9">
         <v>25</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="10">
         <v>6739</v>
       </c>
     </row>
@@ -5916,28 +5984,28 @@
       <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="9">
-        <v>2011</v>
+      <c r="B3" s="11">
+        <v>40834</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>12.5</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="9">
         <v>93.6</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <v>87.6</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>12.5</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>45</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <v>6871</v>
       </c>
     </row>
@@ -5945,28 +6013,28 @@
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="9">
-        <v>2013</v>
+      <c r="B4" s="11">
+        <v>41572</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>7</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>73</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>77</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>12.5</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="9">
         <v>41.5</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>25017</v>
       </c>
     </row>
@@ -5974,34 +6042,29 @@
       <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="9">
-        <v>2015</v>
+      <c r="B5" s="11">
+        <v>42178</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>7.5</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <v>80.599999999999994</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>66.3</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <v>17</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <v>51.5</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <v>27406</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D8" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final visual polish and definitive release
Applied final color palette alignment across all charts to deliver the completed and definitive version of the Excel project.
</commit_message>
<xml_diff>
--- a/arkham-games-dataset.xlsx
+++ b/arkham-games-dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a35c853927159e38/Desktop/Projetos de Análise de Dados/Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="580" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CCC6037-F89E-4F31-8AB6-20E34591E013}"/>
+  <xr:revisionPtr revIDLastSave="611" documentId="8_{CF8A89EB-4A26-4685-8BAF-4BD7872FF1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BDFD054-09AE-4BBE-8CBE-297E6400984C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{D6B36053-BC7E-4879-83CB-ED370B1714CD}"/>
   </bookViews>
@@ -208,7 +208,7 @@
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -481,8 +481,8 @@
   <colors>
     <mruColors>
       <color rgb="FF8B1E2D"/>
+      <color rgb="FF1E3F5A"/>
       <color rgb="FF26382F"/>
-      <color rgb="FF1E3F5A"/>
       <color rgb="FF090A0C"/>
       <color rgb="FFD94A11"/>
       <color rgb="FFE65100"/>
@@ -539,7 +539,7 @@
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="50000">
-                  <a:srgbClr val="8B1E2D"/>
+                  <a:srgbClr val="1E3F5A"/>
                 </a:gs>
               </a:gsLst>
               <a:lin ang="5400000" scaled="1"/>
@@ -568,29 +568,6 @@
             <c:idx val="1"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:gradFill>
-                <a:gsLst>
-                  <a:gs pos="100000">
-                    <a:schemeClr val="bg1">
-                      <a:lumMod val="50000"/>
-                    </a:schemeClr>
-                  </a:gs>
-                  <a:gs pos="50000">
-                    <a:srgbClr val="8B1E2D"/>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000" scaled="1"/>
-              </a:gradFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst>
-                <a:softEdge rad="0"/>
-              </a:effectLst>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000000D-6451-4E07-A78D-57DE91B08B7F}"/>
@@ -777,7 +754,7 @@
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="50000">
-                  <a:srgbClr val="1E3F5A"/>
+                  <a:srgbClr val="8B1E2D"/>
                 </a:gs>
               </a:gsLst>
               <a:lin ang="5400000" scaled="1"/>
@@ -803,7 +780,7 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
@@ -834,7 +811,7 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
@@ -865,7 +842,7 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
@@ -896,7 +873,7 @@
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="50000">
-                    <a:srgbClr val="1E3F5A"/>
+                    <a:srgbClr val="8B1E2D"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="1"/>
@@ -1233,7 +1210,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -1830,7 +1807,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1885,7 +1862,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -1972,7 +1949,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="8B1E2D"/>
+                <a:srgbClr val="1E3F5A"/>
               </a:solidFill>
               <a:ln w="19050">
                 <a:solidFill>
@@ -1992,7 +1969,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="1E3F5A"/>
+                <a:srgbClr val="8B1E2D"/>
               </a:solidFill>
               <a:ln w="19050">
                 <a:solidFill>
@@ -2131,7 +2108,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:ln>
                 <a:noFill/>
               </a:ln>
@@ -2487,7 +2464,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2503,7 +2480,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="bg1"/>
                 </a:solidFill>

</xml_diff>